<commit_message>
Zdjęcia 14 flakonów od właściciela i lista przed publikacją po odpowiedziach
- dev/zdjecia/zdjecia_wlasciciela.py: pliki z Dysku właściciela przypisane do id,
  małe źródła powiększone EDSR x2 (p04, p51, p54 dwa razy), jasne tło wyczyszczone
  do bieli albo przezroczystości (bez tego na karcie zostawał prostokąt wokół flakonu).
- ujednolic_zdjecia.py łączy raport.csv z kolejnych przebiegów zamiast go nadpisywać.
- Karty p01 do p05, p42, p43, p51, p53 do p55, p63 do p65 ze zdjęciami; arkusz importu,
  plik do weryfikacji (119 wierszy) i atrapa katalogu wygenerowane od nowa.
- p52 bez zdjęcia: przysłany plik to Sauvage Eau de Parfum, nie Parfum.
- docs: decyzje 46 do 54, lista przed publikacją z tym, co zostało, raport końcowy
  i plan grafik zaktualizowane.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vr3aaGiTkwi36SuxXxU5aS
</commit_message>
<xml_diff>
--- a/dev/dane/import-do-arkusza.xlsx
+++ b/dev/dane/import-do-arkusza.xlsx
@@ -620,7 +620,11 @@
           <t>p46, p45, p06, p03</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>/img/produkty/p01-800.webp</t>
+        </is>
+      </c>
       <c r="V2" t="n">
         <v>1</v>
       </c>
@@ -711,7 +715,11 @@
           <t>p03, p21, p07</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>/img/produkty/p02-800.webp</t>
+        </is>
+      </c>
       <c r="V3" t="n">
         <v>2</v>
       </c>
@@ -806,7 +814,11 @@
           <t>p02, p08, p21</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>/img/produkty/p03-800.webp</t>
+        </is>
+      </c>
       <c r="V4" t="n">
         <v>3</v>
       </c>
@@ -901,7 +913,11 @@
           <t>p05, p32, p19, p17</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>/img/produkty/p04-800.webp</t>
+        </is>
+      </c>
       <c r="V5" t="n">
         <v>4</v>
       </c>
@@ -996,7 +1012,11 @@
           <t>p04, p19, p17</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>/img/produkty/p05-800.webp</t>
+        </is>
+      </c>
       <c r="V6" t="n">
         <v>5</v>
       </c>
@@ -4591,7 +4611,11 @@
           <t>p10, p35, p70</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr"/>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>/img/produkty/p42-800.webp</t>
+        </is>
+      </c>
       <c r="V43" t="n">
         <v>42</v>
       </c>
@@ -4686,7 +4710,11 @@
           <t>p42, p40, p08</t>
         </is>
       </c>
-      <c r="U44" t="inlineStr"/>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>/img/produkty/p43-800.webp</t>
+        </is>
+      </c>
       <c r="V44" t="n">
         <v>43</v>
       </c>
@@ -5458,7 +5486,11 @@
           <t>p14, p06, p62</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr"/>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>/img/produkty/p51-800.webp</t>
+        </is>
+      </c>
       <c r="V52" t="n">
         <v>51</v>
       </c>
@@ -5644,7 +5676,11 @@
           <t>p54, p52, p11, p70</t>
         </is>
       </c>
-      <c r="U54" t="inlineStr"/>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>/img/produkty/p53-800.webp</t>
+        </is>
+      </c>
       <c r="V54" t="n">
         <v>53</v>
       </c>
@@ -5739,7 +5775,11 @@
           <t>p53, p38, p05, p41</t>
         </is>
       </c>
-      <c r="U55" t="inlineStr"/>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>/img/produkty/p54-800.webp</t>
+        </is>
+      </c>
       <c r="V55" t="n">
         <v>54</v>
       </c>
@@ -5832,7 +5872,11 @@
           <t>p08, p09</t>
         </is>
       </c>
-      <c r="U56" t="inlineStr"/>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>/img/produkty/p55-800.webp</t>
+        </is>
+      </c>
       <c r="V56" t="n">
         <v>55</v>
       </c>
@@ -6502,7 +6546,11 @@
           <t>p44, p52, p10</t>
         </is>
       </c>
-      <c r="U64" t="inlineStr"/>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>/img/produkty/p63-800.webp</t>
+        </is>
+      </c>
       <c r="V64" t="n">
         <v>63</v>
       </c>
@@ -6595,7 +6643,11 @@
           <t>p63, p33, p52</t>
         </is>
       </c>
-      <c r="U65" t="inlineStr"/>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>/img/produkty/p64-800.webp</t>
+        </is>
+      </c>
       <c r="V65" t="n">
         <v>64</v>
       </c>
@@ -6688,7 +6740,11 @@
           <t>p44, p11, p45</t>
         </is>
       </c>
-      <c r="U66" t="inlineStr"/>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>/img/produkty/p65-800.webp</t>
+        </is>
+      </c>
       <c r="V66" t="n">
         <v>65</v>
       </c>
@@ -7527,7 +7583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F134"/>
+  <dimension ref="A1:F120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7593,24 +7649,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>p01</t>
+          <t>p02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Louis Vuitton Imagination</t>
+          <t>Louis Vuitton Pacific Chill</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+          <t>sezon</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Lato (upały), późna wiosna</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>wiosna, lato</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
@@ -7627,166 +7691,182 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>podobne</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Lato (upały), późna wiosna</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>wiosna, lato</t>
-        </is>
-      </c>
+          <t>Xerjoff Renaissance -&gt; renaissance</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>p02</t>
+          <t>p03</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Louis Vuitton Pacific Chill</t>
+          <t>Louis Vuitton Afternoon Swim</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>podobne</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Xerjoff Renaissance -&gt; renaissance</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>pewność danych: średnia</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>bez zmian</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>p02</t>
+          <t>p05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Louis Vuitton Pacific Chill</t>
+          <t>Louis Vuitton Ombre Nomade</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Agarowo-różana</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>orientalna</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>p03</t>
+          <t>p05</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Louis Vuitton Afternoon Swim</t>
+          <t>Louis Vuitton Ombre Nomade</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>podobne</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>bez zmian</t>
-        </is>
-      </c>
+          <t>Amouage Otlands -&gt; otlands</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>p03</t>
+          <t>p06</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Louis Vuitton Afternoon Swim</t>
+          <t>Xerjoff Torino21</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+          <t>podobne</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Xerjoff Renaissance -&gt; renaissance</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>p04</t>
+          <t>p07</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Louis Vuitton Nouveau Monde</t>
+          <t>Xerjoff Renaissance (XJ 1861)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
+          <t>sezon</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Wiosna, lato, wczesna jesień</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>wiosna, lato, jesień</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>p05</t>
+          <t>p08</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Louis Vuitton Ombre Nomade</t>
+          <t>Xerjoff Erba Pura</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -7796,12 +7876,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Agarowo-różana</t>
+          <t>Owocowo-ambrowa</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>orientalna</t>
+          <t>ambrowa</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -7813,568 +7893,584 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>p05</t>
+          <t>p08</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Louis Vuitton Ombre Nomade</t>
+          <t>Xerjoff Erba Pura</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>podobne</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Amouage Otlands -&gt; otlands</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+          <t>Cały rok, najlepiej wiosna i lato</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>wiosna, lato, jesień, zima</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>p05</t>
+          <t>p09</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Louis Vuitton Ombre Nomade</t>
+          <t>Xerjoff Uden</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+          <t>sezon</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Jesień, zima, wczesna wiosna</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>wiosna, jesień, zima</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>p06</t>
+          <t>p09</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Xerjoff Torino21</t>
+          <t>Xerjoff Uden</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>podobne</t>
+          <t>pora</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Xerjoff Renaissance -&gt; renaissance</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
+          <t>Wieczór, chłodny dzień</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>uniwersalna</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>uproszczono do: dzień, wieczór, uniwersalna</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>p07</t>
+          <t>p11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Xerjoff Renaissance (XJ 1861)</t>
+          <t>Creed Aventus</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Wiosna, lato, wczesna jesień</t>
+          <t>Owocowo-drzewna</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>wiosna, lato, jesień</t>
+          <t>drzewna</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>p08</t>
+          <t>p11</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Xerjoff Erba Pura</t>
+          <t>Creed Aventus</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Owocowo-ambrowa</t>
+          <t>Cały rok, najlepiej wiosna i jesień</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ambrowa</t>
+          <t>wiosna, lato, jesień, zima</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>p08</t>
+          <t>p12</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Xerjoff Erba Pura</t>
+          <t>Creed Absolu Aventus</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Cały rok, najlepiej wiosna i lato</t>
+          <t>pewność danych: średnia</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>wiosna, lato, jesień, zima</t>
+          <t>bez zmian</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>p09</t>
+          <t>p12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Xerjoff Uden</t>
+          <t>Creed Absolu Aventus</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Jesień, zima, wczesna wiosna</t>
+          <t>owocowo-drzewna</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>wiosna, jesień, zima</t>
+          <t>drzewna</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>p09</t>
+          <t>p13</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Xerjoff Uden</t>
+          <t>Creed Virgin Island Water</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>pora</t>
+          <t>nazwa</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Wieczór, chłodny dzień</t>
+          <t>Virgin Island Water</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>uniwersalna</t>
+          <t>Virgin Island Water</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>uproszczono do: dzień, wieczór, uniwersalna</t>
+          <t>nazwa do potwierdzenia (w ofercie „Virgin Mountain Water”)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>p11</t>
+          <t>p13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Creed Aventus</t>
+          <t>Creed Virgin Island Water</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>ml_dostepne</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Owocowo-drzewna</t>
+          <t>NIEDOSTĘPNY</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>drzewna</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>niedostępny w źródle; karta pokaże „Wyprzedane” i podobne</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>p11</t>
+          <t>p14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Creed Aventus</t>
+          <t>Creed Silver Mountain Water</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Cały rok, najlepiej wiosna i jesień</t>
+          <t>zielono-herbaciana</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>wiosna, lato, jesień, zima</t>
+          <t>świeża</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>p12</t>
+          <t>p14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Creed Absolu Aventus</t>
+          <t>Creed Silver Mountain Water</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>podobne</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>bez zmian</t>
-        </is>
-      </c>
+          <t>Xerjoff Renaissance -&gt; renaissance</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>p12</t>
+          <t>p15</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Creed Absolu Aventus</t>
+          <t>Amouage Search</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>owocowo-drzewna</t>
+          <t>Wiosna, jesień (uniwersalny)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>drzewna</t>
+          <t>wiosna, jesień</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>p13</t>
+          <t>p15</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Creed Virgin Island Water</t>
+          <t>Amouage Search</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>nazwa</t>
+          <t>ceny</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Virgin Island Water</t>
+          <t>5 ml – 120 zł | 10 ml – 220 zł | 20 ml – 400 zł (promocja)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Virgin Island Water</t>
+          <t>5 ml 120 zł | 10 ml 220 zł | 20 ml 400 zł</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>nazwa do potwierdzenia (w ofercie „Virgin Mountain Water”)</t>
+          <t>cena oznaczona jako promocja; API nie ma pola na starą cenę, pokażemy ją jako zwykłą</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>p13</t>
+          <t>p16</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Creed Virgin Island Water</t>
+          <t>Amouage Reflection Man</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ml_dostepne</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>NIEDOSTĘPNY</t>
+          <t>Cały rok, najlepiej wiosna i jesień</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>wiosna, lato, jesień, zima</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>niedostępny w źródle; karta pokaże „Wyprzedane” i podobne</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>p14</t>
+          <t>p18</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Creed Silver Mountain Water</t>
+          <t>Amouage Interlude Black Iris</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>aktywny</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>zielono-herbaciana</t>
+          <t>pewność danych: niska</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>świeża</t>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>instrukcja arkusza: nie publikować bez weryfikacji piramidy nut</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>p14</t>
+          <t>p18</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Creed Silver Mountain Water</t>
+          <t>Amouage Interlude Black Iris</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>podobne</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Xerjoff Renaissance -&gt; renaissance</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
+          <t>Irysowo-kadzidlana</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>kwiatowa</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>p15</t>
+          <t>p18</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Amouage Search</t>
+          <t>Amouage Interlude Black Iris</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>ml_dostepne</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Wiosna, jesień (uniwersalny)</t>
+          <t>NIEDOSTĘPNY</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>wiosna, jesień</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>niedostępny w źródle; karta pokaże „Wyprzedane” i podobne</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>p15</t>
+          <t>p19</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Amouage Search</t>
+          <t>Amouage Interlude Man</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ceny</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>5 ml – 120 zł | 10 ml – 220 zł | 20 ml – 400 zł (promocja)</t>
+          <t>Dymno-żywiczna</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>5 ml 120 zł | 10 ml 220 zł | 20 ml 400 zł</t>
+          <t>drzewna</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>cena oznaczona jako promocja; API nie ma pola na starą cenę, pokażemy ją jako zwykłą</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>p16</t>
+          <t>p19</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Amouage Reflection Man</t>
+          <t>Amouage Interlude Man</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -8384,12 +8480,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Cały rok, najlepiej wiosna i jesień</t>
+          <t>Zima, późna jesień</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>wiosna, lato, jesień, zima</t>
+          <t>jesień, zima</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -8401,232 +8497,232 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>p18</t>
+          <t>p21</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Amouage Interlude Black Iris</t>
+          <t>Mancera Lemon Line</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>aktywny</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>pewność danych: niska</t>
+          <t>pewność danych: średnia</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>NIE</t>
+          <t>bez zmian</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: nie publikować bez weryfikacji piramidy nut</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>p18</t>
+          <t>p21</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amouage Interlude Black Iris</t>
+          <t>Mancera Lemon Line</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>podobne</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Irysowo-kadzidlana</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>kwiatowa</t>
-        </is>
-      </c>
+          <t>Xerjoff Renaissance -&gt; renaissance</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>p18</t>
+          <t>p24</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Amouage Interlude Black Iris</t>
+          <t>Mancera Tonka Cola</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ml_dostepne</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>NIEDOSTĘPNY</t>
+          <t>pewność danych: średnia</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>bez zmian</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>niedostępny w źródle; karta pokaże „Wyprzedane” i podobne</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>p19</t>
+          <t>p25</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Amouage Interlude Man</t>
+          <t>Mancera Red Tobacco</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Dymno-żywiczna</t>
+          <t>pewność danych: średnia</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>drzewna</t>
+          <t>bez zmian</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>p19</t>
+          <t>p25</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Amouage Interlude Man</t>
+          <t>Mancera Red Tobacco</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Zima, późna jesień</t>
+          <t>Korzenna</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>jesień, zima</t>
+          <t>orientalna</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>p21</t>
+          <t>p26</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Mancera Lemon Line</t>
+          <t>Mancera Instant Crush</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>aktywny</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
+          <t>pewność danych: niska</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>bez zmian</t>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>instrukcja arkusza: nie publikować bez weryfikacji piramidy nut</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>p21</t>
+          <t>p26</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Mancera Lemon Line</t>
+          <t>Mancera Instant Crush</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>podobne</t>
+          <t>ml_dostepne</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Xerjoff Renaissance -&gt; renaissance</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr"/>
+          <t>NIEDOSTĘPNY</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>niedostępny w źródle; karta pokaże „Wyprzedane” i podobne</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>p24</t>
+          <t>p30</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Mancera Tonka Cola</t>
+          <t>Montale Honey Aoud</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -8653,108 +8749,100 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>p25</t>
+          <t>p31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Mancera Red Tobacco</t>
+          <t>Montale Intense Pepper</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>podobne</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>bez zmian</t>
-        </is>
-      </c>
+          <t>Amouage Reflection -&gt; reflection</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>p25</t>
+          <t>p32</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Mancera Red Tobacco</t>
+          <t>Tom Ford Ombré Leather</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>podobne</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Korzenna</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>orientalna</t>
-        </is>
-      </c>
+          <t>LV Nouvau Monde -&gt; nouvau monde</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>p26</t>
+          <t>p33</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Mancera Instant Crush</t>
+          <t>Tom Ford Noir Extreme</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>aktywny</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>pewność danych: niska</t>
+          <t>Korzenno-gourmand</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>NIE</t>
+          <t>gourmand</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: nie publikować bez weryfikacji piramidy nut</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>p26</t>
+          <t>p34</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Mancera Instant Crush</t>
+          <t>Tom Ford Lost Cherry</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -8781,536 +8869,544 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>p30</t>
+          <t>p35</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Montale Honey Aoud</t>
+          <t>Tom Ford Tobacco Vanille</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
+          <t>Korzenno-gourmand</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>bez zmian</t>
+          <t>gourmand</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>p31</t>
+          <t>p36</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Montale Intense Pepper</t>
+          <t>Tom Ford Bois Pacifique</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>podobne</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Amouage Reflection -&gt; reflection</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr"/>
+          <t>Jesień, zima, wczesna wiosna</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>wiosna, jesień, zima</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>p32</t>
+          <t>p37</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Tom Ford Ombré Leather</t>
+          <t>Tom Ford Oud Wood</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>podobne</t>
+          <t>ml_dostepne</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>LV Nouvau Monde -&gt; nouvau monde</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr"/>
+          <t>NIEDOSTĘPNY</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>niedostępny w źródle; karta pokaże „Wyprzedane” i podobne</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>p33</t>
+          <t>p38</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Tom Ford Noir Extreme</t>
+          <t>Tom Ford Ébène Fumé</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Korzenno-gourmand</t>
+          <t>pewność danych: średnia</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>gourmand</t>
+          <t>bez zmian</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>p34</t>
+          <t>p38</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Tom Ford Lost Cherry</t>
+          <t>Tom Ford Ébène Fumé</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ml_dostepne</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>NIEDOSTĘPNY</t>
+          <t>Dymno-drzewna</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>drzewna</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>niedostępny w źródle; karta pokaże „Wyprzedane” i podobne</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>p35</t>
+          <t>p39</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Tom Ford Tobacco Vanille</t>
+          <t>Marc-Antoine Barrois Ganymede</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Korzenno-gourmand</t>
+          <t>Wiosna, jesień (uniwersalny)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>gourmand</t>
+          <t>wiosna, jesień</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>p36</t>
+          <t>p39</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Tom Ford Bois Pacifique</t>
+          <t>Marc-Antoine Barrois Ganymede</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>ceny</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Jesień, zima, wczesna wiosna</t>
+          <t>5 ml – 70 zł | 10 ml – 140 zł (?) | 20 ml – 250 zł</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>wiosna, jesień, zima</t>
+          <t>5 ml 70 zł | 20 ml 250 zł</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>cena 10 ml oznaczona w źródle jako niepewna "(?)", wariant pominięty do potwierdzenia</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>p37</t>
+          <t>p40</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Tom Ford Oud Wood</t>
+          <t>Tiziana Terenzi Kirke</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ml_dostepne</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>NIEDOSTĘPNY</t>
+          <t>Cały rok, najlepiej wiosna i jesień</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>wiosna, lato, jesień, zima</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>niedostępny w źródle; karta pokaże „Wyprzedane” i podobne</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>p38</t>
+          <t>p41</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Tom Ford Ébène Fumé</t>
+          <t>Maison Crivelli Oud Maracujá</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
+          <t>Owocowo-agarowa</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>bez zmian</t>
+          <t>słodka</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>p38</t>
+          <t>p41</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Tom Ford Ébène Fumé</t>
+          <t>Maison Crivelli Oud Maracujá</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Dymno-drzewna</t>
+          <t>Jesień, zima, chłodna wiosna</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>drzewna</t>
+          <t>wiosna, jesień, zima</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>p39</t>
+          <t>p41</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Marc-Antoine Barrois Ganymede</t>
+          <t>Maison Crivelli Oud Maracujá</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>podobne</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Wiosna, jesień (uniwersalny)</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>wiosna, jesień</t>
-        </is>
-      </c>
+          <t>LV Nouvau Monde -&gt; nouvau monde</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>p39</t>
+          <t>p43</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Marc-Antoine Barrois Ganymede</t>
+          <t>Maison Francis Kurkdjian Baccarat Rouge 540</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ceny</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>5 ml – 70 zł | 10 ml – 140 zł (?) | 20 ml – 250 zł</t>
+          <t>Cały rok, najlepiej jesień i zima</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>5 ml 70 zł | 20 ml 250 zł</t>
+          <t>wiosna, lato, jesień, zima</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>cena 10 ml oznaczona w źródle jako niepewna "(?)", wariant pominięty do potwierdzenia</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>p40</t>
+          <t>p43</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Tiziana Terenzi Kirke</t>
+          <t>Maison Francis Kurkdjian Baccarat Rouge 540</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>pora</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Cały rok, najlepiej wiosna i jesień</t>
+          <t>Wieczór (działa też w dzień)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>wiosna, lato, jesień, zima</t>
+          <t>uniwersalna</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>uproszczono do: dzień, wieczór, uniwersalna</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>p41</t>
+          <t>p44</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Maison Crivelli Oud Maracujá</t>
+          <t>Essential Parfums Bois Impérial</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>podobne</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Owocowo-agarowa</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>słodka</t>
-        </is>
-      </c>
+          <t>Nous Tous Saffrano Absolu -&gt; saffrano absolu</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>p41</t>
+          <t>p47</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Maison Crivelli Oud Maracujá</t>
+          <t>Nous Tous Secco di Como</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>podobne</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Jesień, zima, chłodna wiosna</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>wiosna, jesień, zima</t>
-        </is>
-      </c>
+          <t>Xerjoff Renaissance -&gt; renaissance</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>p41</t>
+          <t>p48</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Maison Crivelli Oud Maracujá</t>
+          <t>Nous Tous Aurora Siciliana</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>podobne</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>LV Nouvau Monde -&gt; nouvau monde</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr"/>
+          <t>Owocowo-kwiatowa</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>kwiatowa</t>
+        </is>
+      </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>p42</t>
+          <t>p50</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Maison Francis Kurkdjian Grand Soir</t>
+          <t>Nous Tous Milano 3AM</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>korzenna</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>orientalna</t>
+        </is>
+      </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>p43</t>
+          <t>p50</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Maison Francis Kurkdjian Baccarat Rouge 540</t>
+          <t>Nous Tous Milano 3AM</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -9320,7 +9416,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Cały rok, najlepiej jesień i zima</t>
+          <t>Cały rok, najlepiej chłodne wieczory</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -9337,244 +9433,220 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>p43</t>
+          <t>p52</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Maison Francis Kurkdjian Baccarat Rouge 540</t>
+          <t>Dior Sauvage Parfum</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>pora</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Wieczór (działa też w dzień)</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>uniwersalna</t>
-        </is>
-      </c>
+          <t>zdjecie_url</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>uproszczono do: dzień, wieczór, uniwersalna</t>
+          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>p43</t>
+          <t>p53</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Maison Francis Kurkdjian Baccarat Rouge 540</t>
+          <t>Dior Sauvage Elixir</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Korzenno-ambrowa</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ambrowa</t>
+        </is>
+      </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>p44</t>
+          <t>p55</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Essential Parfums Bois Impérial</t>
+          <t>Versace Eros Parfum</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>podobne</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Nous Tous Saffrano Absolu -&gt; saffrano absolu</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr"/>
+          <t>pewność danych: średnia</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>bez zmian</t>
+        </is>
+      </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>p47</t>
+          <t>p56</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Nous Tous Secco di Como</t>
+          <t>wiersz Lp. 56 (bez nazwy)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>podobne</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Xerjoff Renaissance -&gt; renaissance</t>
-        </is>
-      </c>
+          <t>marka, nazwa</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>brak marki i nazwy; pozycja wyłączona do czasu uzupełnienia</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>p48</t>
+          <t>p56</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Nous Tous Aurora Siciliana</t>
+          <t>wiersz Lp. 56 (bez nazwy)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Owocowo-kwiatowa</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>kwiatowa</t>
-        </is>
-      </c>
+          <t>sezon</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>brak w źródle</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>p50</t>
+          <t>p56</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Nous Tous Milano 3AM</t>
+          <t>wiersz Lp. 56 (bez nazwy)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>korzenna</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>orientalna</t>
-        </is>
-      </c>
+          <t>pora</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>brak w źródle</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>p50</t>
+          <t>p56</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Nous Tous Milano 3AM</t>
+          <t>wiersz Lp. 56 (bez nazwy)</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>sezon</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Cały rok, najlepiej chłodne wieczory</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>wiosna, lato, jesień, zima</t>
-        </is>
-      </c>
+          <t>trwalosc</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>brak w źródle</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>p51</t>
+          <t>p56</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Dior Homme Cologne</t>
+          <t>wiersz Lp. 56 (bez nazwy)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
+          <t>projekcja</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>brak w źródle</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>p52</t>
+          <t>p56</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Dior Sauvage Parfum</t>
+          <t>wiersz Lp. 56 (bez nazwy)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -9593,225 +9665,217 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>p53</t>
+          <t>p57</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Dior Sauvage Elixir</t>
+          <t>wiersz Lp. 57 (bez nazwy)</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Korzenno-ambrowa</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>ambrowa</t>
-        </is>
-      </c>
+          <t>marka, nazwa</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>brak marki i nazwy; pozycja wyłączona do czasu uzupełnienia</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>p53</t>
+          <t>p57</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Dior Sauvage Elixir</t>
+          <t>wiersz Lp. 57 (bez nazwy)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Korzenno-drzewna</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>drzewna</t>
+        </is>
+      </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>p54</t>
+          <t>p57</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Dior Sauvage Extrait</t>
+          <t>wiersz Lp. 57 (bez nazwy)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>brak w źródle</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>p55</t>
+          <t>p57</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Versace Eros Parfum</t>
+          <t>wiersz Lp. 57 (bez nazwy)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>pewność danych: średnia</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>bez zmian</t>
-        </is>
-      </c>
+          <t>pora</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>brak w źródle</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>p55</t>
+          <t>p57</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Versace Eros Parfum</t>
+          <t>wiersz Lp. 57 (bez nazwy)</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
+          <t>trwalosc</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>brak w źródle</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>p56</t>
+          <t>p57</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>wiersz Lp. 56 (bez nazwy)</t>
+          <t>wiersz Lp. 57 (bez nazwy)</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>marka, nazwa</t>
+          <t>projekcja</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>brak marki i nazwy; pozycja wyłączona do czasu uzupełnienia</t>
+          <t>brak w źródle</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>p56</t>
+          <t>p57</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>wiersz Lp. 56 (bez nazwy)</t>
+          <t>wiersz Lp. 57 (bez nazwy)</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>zdjecie_url</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>brak w źródle</t>
+          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>p56</t>
+          <t>p58</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>wiersz Lp. 56 (bez nazwy)</t>
+          <t>wiersz Lp. 58 (bez nazwy)</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>pora</t>
+          <t>marka, nazwa</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
-          <t>brak w źródle</t>
+          <t>brak marki i nazwy; pozycja wyłączona do czasu uzupełnienia</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>p56</t>
+          <t>p58</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>wiersz Lp. 56 (bez nazwy)</t>
+          <t>wiersz Lp. 58 (bez nazwy)</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>trwalosc</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -9825,17 +9889,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>p56</t>
+          <t>p58</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>wiersz Lp. 56 (bez nazwy)</t>
+          <t>wiersz Lp. 58 (bez nazwy)</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>projekcja</t>
+          <t>pora</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
@@ -9849,380 +9913,452 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>p56</t>
+          <t>p58</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>wiersz Lp. 56 (bez nazwy)</t>
+          <t>wiersz Lp. 58 (bez nazwy)</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
+          <t>trwalosc</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>brak w źródle</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>p57</t>
+          <t>p58</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>wiersz Lp. 57 (bez nazwy)</t>
+          <t>wiersz Lp. 58 (bez nazwy)</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>marka, nazwa</t>
+          <t>projekcja</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>brak marki i nazwy; pozycja wyłączona do czasu uzupełnienia</t>
+          <t>brak w źródle</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>p57</t>
+          <t>p58</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>wiersz Lp. 57 (bez nazwy)</t>
+          <t>wiersz Lp. 58 (bez nazwy)</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Korzenno-drzewna</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>drzewna</t>
-        </is>
-      </c>
+          <t>ceny</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>brak cen</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>p57</t>
+          <t>p58</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>wiersz Lp. 57 (bez nazwy)</t>
+          <t>wiersz Lp. 58 (bez nazwy)</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>zdjecie_url</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
-          <t>brak w źródle</t>
+          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>p57</t>
+          <t>p59</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>wiersz Lp. 57 (bez nazwy)</t>
+          <t>Hugo Boss Bottled Elixir</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>pora</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr"/>
+          <t>nuty / osiągi</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>pewność danych: średnia</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>bez zmian</t>
+        </is>
+      </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>brak w źródle</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>p57</t>
+          <t>p59</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>wiersz Lp. 57 (bez nazwy)</t>
+          <t>Hugo Boss Bottled Elixir</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>trwalosc</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr"/>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Korzenno-drzewna</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>drzewna</t>
+        </is>
+      </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>brak w źródle</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>p57</t>
+          <t>p60</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>wiersz Lp. 57 (bez nazwy)</t>
+          <t>Hugo Boss Bottled Absolu</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>projekcja</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr"/>
-      <c r="E85" t="inlineStr"/>
+          <t>aktywny</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>pewność danych: niska</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>brak w źródle</t>
+          <t>instrukcja arkusza: nie publikować bez weryfikacji piramidy nut</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>p57</t>
+          <t>p60</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>wiersz Lp. 57 (bez nazwy)</t>
+          <t>Hugo Boss Bottled Absolu</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr"/>
-      <c r="E86" t="inlineStr"/>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Korzenno-gourmand</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>gourmand</t>
+        </is>
+      </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>p58</t>
+          <t>p60</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>wiersz Lp. 58 (bez nazwy)</t>
+          <t>Hugo Boss Bottled Absolu</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>marka, nazwa</t>
+          <t>zdjecie_url</t>
         </is>
       </c>
       <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
-          <t>brak marki i nazwy; pozycja wyłączona do czasu uzupełnienia</t>
+          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>p58</t>
+          <t>p61</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>wiersz Lp. 58 (bez nazwy)</t>
+          <t>Hugo Boss Bottled Beyond</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>sezon</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr"/>
+          <t>nuty / osiągi</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>pewność danych: średnia</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>bez zmian</t>
+        </is>
+      </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>brak w źródle</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>p58</t>
+          <t>p63</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>wiersz Lp. 58 (bez nazwy)</t>
+          <t>YSL Y Parfum</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>pora</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr"/>
-      <c r="E89" t="inlineStr"/>
+          <t>nuty / osiągi</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>pewność danych: średnia</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>bez zmian</t>
+        </is>
+      </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>brak w źródle</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>p58</t>
+          <t>p63</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>wiersz Lp. 58 (bez nazwy)</t>
+          <t>YSL Y Parfum</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>trwalosc</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr"/>
+          <t>sezon</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Cały rok, najlepiej wiosna i jesień</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>wiosna, lato, jesień, zima</t>
+        </is>
+      </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>brak w źródle</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>p58</t>
+          <t>p64</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>wiersz Lp. 58 (bez nazwy)</t>
+          <t>YSL MYSLF Parfum</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>projekcja</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr"/>
-      <c r="E91" t="inlineStr"/>
+          <t>nuty / osiągi</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>pewność danych: średnia</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>bez zmian</t>
+        </is>
+      </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>brak w źródle</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>p58</t>
+          <t>p65</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>wiersz Lp. 58 (bez nazwy)</t>
+          <t>Hermès Terre d'Hermès Eau Intense Vétiver</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>ceny</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr"/>
-      <c r="E92" t="inlineStr"/>
+          <t>nuty / osiągi</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>pewność danych: średnia</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>bez zmian</t>
+        </is>
+      </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>brak cen</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>p58</t>
+          <t>p65</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>wiersz Lp. 58 (bez nazwy)</t>
+          <t>Hermès Terre d'Hermès Eau Intense Vétiver</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr"/>
+          <t>sezon</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Wiosna, lato, wczesna jesień</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>wiosna, lato, jesień</t>
+        </is>
+      </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>p59</t>
+          <t>p66</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Hugo Boss Bottled Elixir</t>
+          <t>Rabanne Black XS</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -10249,12 +10385,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>p59</t>
+          <t>p66</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Hugo Boss Bottled Elixir</t>
+          <t>Rabanne Black XS</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -10264,12 +10400,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Korzenno-drzewna</t>
+          <t>Korzenno-cytrusowa</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>drzewna</t>
+          <t>cytrusowa</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -10281,100 +10417,108 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>p60</t>
+          <t>p68</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Hugo Boss Bottled Absolu</t>
+          <t>Rabanne One Million</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>aktywny</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>pewność danych: niska</t>
+          <t>Korzenno-słodka</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>NIE</t>
+          <t>słodka</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: nie publikować bez weryfikacji piramidy nut</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>p60</t>
+          <t>p69</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Hugo Boss Bottled Absolu</t>
+          <t>Azzaro Chrome</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Korzenno-gourmand</t>
+          <t>pewność danych: średnia</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>gourmand</t>
+          <t>bez zmian</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>p60</t>
+          <t>p70</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Hugo Boss Bottled Absolu</t>
+          <t>Azzaro Forever Wanted Elixir</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr"/>
+          <t>nuty / osiągi</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>pewność danych: średnia</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>bez zmian</t>
+        </is>
+      </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>p61</t>
+          <t>p71</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Hugo Boss Bottled Beyond</t>
+          <t>Azzaro The Most Wanted Parfum</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -10401,308 +10545,280 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>p63</t>
+          <t>p71</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>YSL Y Parfum</t>
+          <t>Azzaro The Most Wanted Parfum</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
+          <t>Korzenno-drzewna</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>bez zmian</t>
+          <t>drzewna</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>p63</t>
+          <t>z01</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>YSL Y Parfum</t>
+          <t>LV DISCOVERY SET</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>sezon</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>Cały rok, najlepiej wiosna i jesień</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>wiosna, lato, jesień, zima</t>
-        </is>
-      </c>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>p63</t>
+          <t>z01</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>YSL Y Parfum</t>
+          <t>LV DISCOVERY SET</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
+          <t>opis</t>
         </is>
       </c>
       <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>p64</t>
+          <t>z02</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>YSL MYSLF Parfum</t>
+          <t>XERJOFF DISCOVERY SET</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>sklad</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
+          <t>5 × 5 ml (do ustalenia skład, sugerowane: Torino21, Renaissance, Erba Pura, Uden, Naxos)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>bez zmian</t>
+          <t>p06:5, p07:5, p08:5, p09:5, p10:5</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>skład „do ustalenia”; wpisano propozycję ze źródła, zestaw wyłączony</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>p64</t>
+          <t>z02</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>YSL MYSLF Parfum</t>
+          <t>XERJOFF DISCOVERY SET</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr"/>
+          <t>sklad</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Renaissance -&gt; renaissance</t>
+        </is>
+      </c>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>p65</t>
+          <t>z02</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Hermès Terre d'Hermès Eau Intense Vétiver</t>
+          <t>XERJOFF DISCOVERY SET</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>pewność danych: średnia</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>bez zmian</t>
-        </is>
-      </c>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>p65</t>
+          <t>z02</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Hermès Terre d'Hermès Eau Intense Vétiver</t>
+          <t>XERJOFF DISCOVERY SET</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>sezon</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>Wiosna, lato, wczesna jesień</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>wiosna, lato, jesień</t>
-        </is>
-      </c>
+          <t>opis</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>p65</t>
+          <t>z03</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Hermès Terre d'Hermès Eau Intense Vétiver</t>
+          <t>NOUS TOUS DISCOVERY SET</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr"/>
-      <c r="E107" t="inlineStr"/>
+          <t>cena</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>350 zł</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>cena zapisana jako tekst</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>p66</t>
+          <t>z03</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Rabanne Black XS</t>
+          <t>NOUS TOUS DISCOVERY SET</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>pewność danych: średnia</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>bez zmian</t>
-        </is>
-      </c>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>p66</t>
+          <t>z03</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Rabanne Black XS</t>
+          <t>NOUS TOUS DISCOVERY SET</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>Korzenno-cytrusowa</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>cytrusowa</t>
-        </is>
-      </c>
+          <t>opis</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>p68</t>
+          <t>z04</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Rabanne One Million</t>
+          <t>SWEET &amp; SPICY SET</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -10710,239 +10826,203 @@
           <t>rodzina</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>Korzenno-słodka</t>
-        </is>
-      </c>
+      <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr">
         <is>
-          <t>słodka</t>
+          <t>gourmand</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>propozycja z opisu zestawu w źródle (gourmand wprost w treści)</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>p69</t>
+          <t>z04</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Azzaro Chrome</t>
+          <t>SWEET &amp; SPICY SET</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>pewność danych: średnia</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>bez zmian</t>
-        </is>
-      </c>
+          <t>opis</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr"/>
+      <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>p70</t>
+          <t>z05</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Azzaro Forever Wanted Elixir</t>
+          <t>ENTRY SET</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>sklad</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>bez zmian</t>
-        </is>
-      </c>
+          <t>Amouage Reflection -&gt; reflection</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>p71</t>
+          <t>z05</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Azzaro The Most Wanted Parfum</t>
+          <t>ENTRY SET</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>pewność danych: średnia</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>bez zmian</t>
-        </is>
-      </c>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>p71</t>
+          <t>z05</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Azzaro The Most Wanted Parfum</t>
+          <t>ENTRY SET</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>Korzenno-drzewna</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>drzewna</t>
-        </is>
-      </c>
+          <t>opis</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>z01</t>
+          <t>z06</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>LV DISCOVERY SET</t>
+          <t>AUTUMN DISCOVERY SET</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr"/>
+          <t>sklad</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>YSL Y le Parfum -&gt; y le parfum</t>
+        </is>
+      </c>
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>z01</t>
+          <t>z06</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>LV DISCOVERY SET</t>
+          <t>AUTUMN DISCOVERY SET</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>opis</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>z02</t>
+          <t>z06</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>XERJOFF DISCOVERY SET</t>
+          <t>AUTUMN DISCOVERY SET</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>sklad</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>5 × 5 ml (do ustalenia skład, sugerowane: Torino21, Renaissance, Erba Pura, Uden, Naxos)</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>p06:5, p07:5, p08:5, p09:5, p10:5</t>
-        </is>
-      </c>
+          <t>opis</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
-          <t>skład „do ustalenia”; wpisano propozycję ze źródła, zestaw wyłączony</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>z02</t>
+          <t>z07</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>XERJOFF DISCOVERY SET</t>
+          <t>WINTER DISCOVERY SET</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -10952,25 +11032,29 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Renaissance -&gt; renaissance</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr"/>
+          <t>5x ml (BOSS Bottled Absolu, MFK Grand Soir, Maison Crivelli Oud Maracuja, Tom Ford Tobacco Vanille, Montale Arabians Tonka)</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>p60:5, p42:5, p41:5, p35:5, p28:5</t>
+        </is>
+      </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>w źródle „5x ml” bez pojemności; przyjęto 5 ml</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>z02</t>
+          <t>z07</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>XERJOFF DISCOVERY SET</t>
+          <t>WINTER DISCOVERY SET</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -10989,12 +11073,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>z02</t>
+          <t>z07</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>XERJOFF DISCOVERY SET</t>
+          <t>WINTER DISCOVERY SET</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -11005,370 +11089,6 @@
       <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr">
-        <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>z03</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>NOUS TOUS DISCOVERY SET</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>cena</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>350 zł</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>cena zapisana jako tekst</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>z03</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>NOUS TOUS DISCOVERY SET</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr"/>
-      <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>z03</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>NOUS TOUS DISCOVERY SET</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>opis</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr"/>
-      <c r="E123" t="inlineStr"/>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>z04</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>SWEET &amp; SPICY SET</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr"/>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>gourmand</t>
-        </is>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>propozycja z opisu zestawu w źródle (gourmand wprost w treści)</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>z04</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>SWEET &amp; SPICY SET</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>opis</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr"/>
-      <c r="E125" t="inlineStr"/>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>z05</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>ENTRY SET</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>sklad</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>Amouage Reflection -&gt; reflection</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr"/>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>z05</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>ENTRY SET</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr"/>
-      <c r="E127" t="inlineStr"/>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>z05</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>ENTRY SET</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>opis</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr"/>
-      <c r="E128" t="inlineStr"/>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>z06</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>AUTUMN DISCOVERY SET</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>sklad</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>YSL Y le Parfum -&gt; y le parfum</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr"/>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>z06</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>AUTUMN DISCOVERY SET</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr"/>
-      <c r="E130" t="inlineStr"/>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>z06</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>AUTUMN DISCOVERY SET</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>opis</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr"/>
-      <c r="E131" t="inlineStr"/>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>z07</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>WINTER DISCOVERY SET</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>sklad</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>5x ml (BOSS Bottled Absolu, MFK Grand Soir, Maison Crivelli Oud Maracuja, Tom Ford Tobacco Vanille, Montale Arabians Tonka)</t>
-        </is>
-      </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>p60:5, p42:5, p41:5, p35:5, p28:5</t>
-        </is>
-      </c>
-      <c r="F132" t="inlineStr">
-        <is>
-          <t>w źródle „5x ml” bez pojemności; przyjęto 5 ml</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>z07</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>WINTER DISCOVERY SET</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr"/>
-      <c r="E133" t="inlineStr"/>
-      <c r="F133" t="inlineStr">
-        <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>z07</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>WINTER DISCOVERY SET</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>opis</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr"/>
-      <c r="E134" t="inlineStr"/>
-      <c r="F134" t="inlineStr">
         <is>
           <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>

</xml_diff>

<commit_message>
Zdjęcia p51 i p52 od właściciela, bon 50 zł za opóźnienie realizacji
- p52 Dior Sauvage Parfum (etykieta PARFUM, EDSR x2) i nowe p51 Dior Homme Cologne
  (1333 × 2000 px) z plików przysłanych w rozmowie; wszystkie 64 aktywne zapachy mają zdjęcie.
- zdjecia_wlasciciela.py: opcjonalna lista id, przetwarza tylko wskazane zdjęcia
  i podmienia ich wiersze w zrodla-wlasciciel.csv.
- Realizacja dłuższa niż 7 dni roboczych: bon 50 zł na kolejne zakupy od 199 zł
  w gwarancjach, FAQ, regulaminie (punkt 5, z TODO na zasady bonu) i w refs/README.md.
- docs: potwierdzony e-mail i termin 7 dni roboczych, decyzje 55 i 56, lista przed
  publikacją z pytaniami o wykorzystanie bonu.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vr3aaGiTkwi36SuxXxU5aS
</commit_message>
<xml_diff>
--- a/dev/dane/import-do-arkusza.xlsx
+++ b/dev/dane/import-do-arkusza.xlsx
@@ -5583,7 +5583,11 @@
           <t>p53, p54, p11</t>
         </is>
       </c>
-      <c r="U53" t="inlineStr"/>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>/img/produkty/p52-800.webp</t>
+        </is>
+      </c>
       <c r="V53" t="n">
         <v>52</v>
       </c>
@@ -7583,7 +7587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:F119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9433,88 +9437,88 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>p52</t>
+          <t>p53</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Dior Sauvage Parfum</t>
+          <t>Dior Sauvage Elixir</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Korzenno-ambrowa</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ambrowa</t>
+        </is>
+      </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>p53</t>
+          <t>p55</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Dior Sauvage Elixir</t>
+          <t>Versace Eros Parfum</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Korzenno-ambrowa</t>
+          <t>pewność danych: średnia</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ambrowa</t>
+          <t>bez zmian</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>p55</t>
+          <t>p56</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Versace Eros Parfum</t>
+          <t>wiersz Lp. 56 (bez nazwy)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>pewność danych: średnia</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>bez zmian</t>
-        </is>
-      </c>
+          <t>marka, nazwa</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>brak marki i nazwy; pozycja wyłączona do czasu uzupełnienia</t>
         </is>
       </c>
     </row>
@@ -9531,14 +9535,14 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>marka, nazwa</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>brak marki i nazwy; pozycja wyłączona do czasu uzupełnienia</t>
+          <t>brak w źródle</t>
         </is>
       </c>
     </row>
@@ -9555,7 +9559,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>pora</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -9579,7 +9583,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>pora</t>
+          <t>trwalosc</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -9603,7 +9607,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>trwalosc</t>
+          <t>projekcja</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -9627,38 +9631,38 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>projekcja</t>
+          <t>zdjecie_url</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>brak w źródle</t>
+          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>p56</t>
+          <t>p57</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>wiersz Lp. 56 (bez nazwy)</t>
+          <t>wiersz Lp. 57 (bez nazwy)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
+          <t>marka, nazwa</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>brak marki i nazwy; pozycja wyłączona do czasu uzupełnienia</t>
         </is>
       </c>
     </row>
@@ -9675,14 +9679,22 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>marka, nazwa</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Korzenno-drzewna</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>drzewna</t>
+        </is>
+      </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>brak marki i nazwy; pozycja wyłączona do czasu uzupełnienia</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
@@ -9699,22 +9711,14 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Korzenno-drzewna</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>drzewna</t>
-        </is>
-      </c>
+          <t>sezon</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>brak w źródle</t>
         </is>
       </c>
     </row>
@@ -9731,7 +9735,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>pora</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
@@ -9755,7 +9759,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>pora</t>
+          <t>trwalosc</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
@@ -9779,7 +9783,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>trwalosc</t>
+          <t>projekcja</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
@@ -9803,38 +9807,38 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>projekcja</t>
+          <t>zdjecie_url</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>brak w źródle</t>
+          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>p57</t>
+          <t>p58</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>wiersz Lp. 57 (bez nazwy)</t>
+          <t>wiersz Lp. 58 (bez nazwy)</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
+          <t>marka, nazwa</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>brak marki i nazwy; pozycja wyłączona do czasu uzupełnienia</t>
         </is>
       </c>
     </row>
@@ -9851,14 +9855,14 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>marka, nazwa</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
-          <t>brak marki i nazwy; pozycja wyłączona do czasu uzupełnienia</t>
+          <t>brak w źródle</t>
         </is>
       </c>
     </row>
@@ -9875,7 +9879,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>pora</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -9899,7 +9903,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>pora</t>
+          <t>trwalosc</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
@@ -9923,7 +9927,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>trwalosc</t>
+          <t>projekcja</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
@@ -9947,14 +9951,14 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>projekcja</t>
+          <t>ceny</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>brak w źródle</t>
+          <t>brak cen</t>
         </is>
       </c>
     </row>
@@ -9971,38 +9975,46 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ceny</t>
+          <t>zdjecie_url</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>brak cen</t>
+          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>p58</t>
+          <t>p59</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>wiersz Lp. 58 (bez nazwy)</t>
+          <t>Hugo Boss Bottled Elixir</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
+          <t>nuty / osiągi</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>pewność danych: średnia</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>bez zmian</t>
+        </is>
+      </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
@@ -10019,54 +10031,54 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
+          <t>Korzenno-drzewna</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>bez zmian</t>
+          <t>drzewna</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>p59</t>
+          <t>p60</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Hugo Boss Bottled Elixir</t>
+          <t>Hugo Boss Bottled Absolu</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>aktywny</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Korzenno-drzewna</t>
+          <t>pewność danych: niska</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>drzewna</t>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>instrukcja arkusza: nie publikować bez weryfikacji piramidy nut</t>
         </is>
       </c>
     </row>
@@ -10083,22 +10095,22 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>aktywny</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>pewność danych: niska</t>
+          <t>Korzenno-gourmand</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>NIE</t>
+          <t>gourmand</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: nie publikować bez weryfikacji piramidy nut</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
@@ -10115,58 +10127,58 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>Korzenno-gourmand</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>gourmand</t>
-        </is>
-      </c>
+          <t>zdjecie_url</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>p60</t>
+          <t>p61</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Hugo Boss Bottled Absolu</t>
+          <t>Hugo Boss Bottled Beyond</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
+          <t>nuty / osiągi</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>pewność danych: średnia</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>bez zmian</t>
+        </is>
+      </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>p61</t>
+          <t>p63</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Hugo Boss Bottled Beyond</t>
+          <t>YSL Y Parfum</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -10203,66 +10215,66 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
+          <t>Cały rok, najlepiej wiosna i jesień</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>bez zmian</t>
+          <t>wiosna, lato, jesień, zima</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>p63</t>
+          <t>p64</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>YSL Y Parfum</t>
+          <t>YSL MYSLF Parfum</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Cały rok, najlepiej wiosna i jesień</t>
+          <t>pewność danych: średnia</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>wiosna, lato, jesień, zima</t>
+          <t>bez zmian</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>p64</t>
+          <t>p65</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>YSL MYSLF Parfum</t>
+          <t>Hermès Terre d'Hermès Eau Intense Vétiver</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -10299,54 +10311,54 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
+          <t>Wiosna, lato, wczesna jesień</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>bez zmian</t>
+          <t>wiosna, lato, jesień</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>p65</t>
+          <t>p66</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Hermès Terre d'Hermès Eau Intense Vétiver</t>
+          <t>Rabanne Black XS</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Wiosna, lato, wczesna jesień</t>
+          <t>pewność danych: średnia</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>wiosna, lato, jesień</t>
+          <t>bez zmian</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
@@ -10363,34 +10375,34 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
+          <t>Korzenno-cytrusowa</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>bez zmian</t>
+          <t>cytrusowa</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>p66</t>
+          <t>p68</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Rabanne Black XS</t>
+          <t>Rabanne One Million</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -10400,12 +10412,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Korzenno-cytrusowa</t>
+          <t>Korzenno-słodka</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>cytrusowa</t>
+          <t>słodka</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -10417,44 +10429,44 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>p68</t>
+          <t>p69</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Rabanne One Million</t>
+          <t>Azzaro Chrome</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Korzenno-słodka</t>
+          <t>pewność danych: średnia</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>słodka</t>
+          <t>bez zmian</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>p69</t>
+          <t>p70</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Azzaro Chrome</t>
+          <t>Azzaro Forever Wanted Elixir</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -10481,12 +10493,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>p70</t>
+          <t>p71</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Azzaro Forever Wanted Elixir</t>
+          <t>Azzaro The Most Wanted Parfum</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -10523,34 +10535,34 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
+          <t>Korzenno-drzewna</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>bez zmian</t>
+          <t>drzewna</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>p71</t>
+          <t>z01</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Azzaro The Most Wanted Parfum</t>
+          <t>LV DISCOVERY SET</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -10558,19 +10570,11 @@
           <t>rodzina</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>Korzenno-drzewna</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>drzewna</t>
-        </is>
-      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
@@ -10587,38 +10591,46 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>opis</t>
         </is>
       </c>
       <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>z01</t>
+          <t>z02</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>LV DISCOVERY SET</t>
+          <t>XERJOFF DISCOVERY SET</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>opis</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr"/>
-      <c r="E102" t="inlineStr"/>
+          <t>sklad</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>5 × 5 ml (do ustalenia skład, sugerowane: Torino21, Renaissance, Erba Pura, Uden, Naxos)</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>p06:5, p07:5, p08:5, p09:5, p10:5</t>
+        </is>
+      </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
+          <t>skład „do ustalenia”; wpisano propozycję ze źródła, zestaw wyłączony</t>
         </is>
       </c>
     </row>
@@ -10640,17 +10652,13 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>5 × 5 ml (do ustalenia skład, sugerowane: Torino21, Renaissance, Erba Pura, Uden, Naxos)</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>p06:5, p07:5, p08:5, p09:5, p10:5</t>
-        </is>
-      </c>
+          <t>Renaissance -&gt; renaissance</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
-          <t>skład „do ustalenia”; wpisano propozycję ze źródła, zestaw wyłączony</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
@@ -10667,18 +10675,14 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>sklad</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>Renaissance -&gt; renaissance</t>
-        </is>
-      </c>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
@@ -10695,38 +10699,46 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>opis</t>
         </is>
       </c>
       <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>z02</t>
+          <t>z03</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>XERJOFF DISCOVERY SET</t>
+          <t>NOUS TOUS DISCOVERY SET</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>opis</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr"/>
-      <c r="E106" t="inlineStr"/>
+          <t>cena</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>350 zł</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
+          <t>cena zapisana jako tekst</t>
         </is>
       </c>
     </row>
@@ -10743,22 +10755,14 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>cena</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>350 zł</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr"/>
+      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
-          <t>cena zapisana jako tekst</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
@@ -10775,38 +10779,42 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>opis</t>
         </is>
       </c>
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>z03</t>
+          <t>z04</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>NOUS TOUS DISCOVERY SET</t>
+          <t>SWEET &amp; SPICY SET</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>opis</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D109" t="inlineStr"/>
-      <c r="E109" t="inlineStr"/>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>gourmand</t>
+        </is>
+      </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
+          <t>propozycja z opisu zestawu w źródle (gourmand wprost w treści)</t>
         </is>
       </c>
     </row>
@@ -10823,42 +10831,42 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>opis</t>
         </is>
       </c>
       <c r="D110" t="inlineStr"/>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>gourmand</t>
-        </is>
-      </c>
+      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
-          <t>propozycja z opisu zestawu w źródle (gourmand wprost w treści)</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>z04</t>
+          <t>z05</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>SWEET &amp; SPICY SET</t>
+          <t>ENTRY SET</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>opis</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr"/>
+          <t>sklad</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Amouage Reflection -&gt; reflection</t>
+        </is>
+      </c>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
@@ -10875,18 +10883,14 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>sklad</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>Amouage Reflection -&gt; reflection</t>
-        </is>
-      </c>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
@@ -10903,38 +10907,42 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>opis</t>
         </is>
       </c>
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>z05</t>
+          <t>z06</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>ENTRY SET</t>
+          <t>AUTUMN DISCOVERY SET</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>opis</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr"/>
+          <t>sklad</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>YSL Y le Parfum -&gt; y le parfum</t>
+        </is>
+      </c>
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
@@ -10951,18 +10959,14 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>sklad</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>YSL Y le Parfum -&gt; y le parfum</t>
-        </is>
-      </c>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
@@ -10979,38 +10983,46 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>opis</t>
         </is>
       </c>
       <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>z06</t>
+          <t>z07</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>AUTUMN DISCOVERY SET</t>
+          <t>WINTER DISCOVERY SET</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>opis</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr"/>
-      <c r="E117" t="inlineStr"/>
+          <t>sklad</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>5x ml (BOSS Bottled Absolu, MFK Grand Soir, Maison Crivelli Oud Maracuja, Tom Ford Tobacco Vanille, Montale Arabians Tonka)</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>p60:5, p42:5, p41:5, p35:5, p28:5</t>
+        </is>
+      </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
+          <t>w źródle „5x ml” bez pojemności; przyjęto 5 ml</t>
         </is>
       </c>
     </row>
@@ -11027,22 +11039,14 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>sklad</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>5x ml (BOSS Bottled Absolu, MFK Grand Soir, Maison Crivelli Oud Maracuja, Tom Ford Tobacco Vanille, Montale Arabians Tonka)</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>p60:5, p42:5, p41:5, p35:5, p28:5</t>
-        </is>
-      </c>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
-          <t>w źródle „5x ml” bez pojemności; przyjęto 5 ml</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
@@ -11059,36 +11063,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>opis</t>
         </is>
       </c>
       <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
-        <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>z07</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>WINTER DISCOVERY SET</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>opis</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr"/>
-      <c r="E120" t="inlineStr"/>
-      <c r="F120" t="inlineStr">
         <is>
           <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>

</xml_diff>

<commit_message>
Katalog: Bestsellery i Nowości, ostatnie zdjęcia od właściciela (decyzje 77, 78)
- przyciski „Bestsellery” i „Nowości” nad wynikami, sekcja „Wyróżnione”
  w filtrach, chip do usunięcia, link ?pokaz=bestsellery / ?pokaz=nowosci
- pasek katalogu bez nachodzenia przycisku „Filtry” na przełącznik przy
  wąskich ekranach (krótsze etykiety poniżej 30rem, zawijanie zamiast
  nakładania)
- zdjęcia p83 Oud Satin Mood, p98 Wet Cherry Liquor i p81 Ambre Latte od
  właściciela; zdjęcie mają wszystkie 94 aktywne zapachy

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vr3aaGiTkwi36SuxXxU5aS
</commit_message>
<xml_diff>
--- a/dev/dane/import-do-arkusza.xlsx
+++ b/dev/dane/import-do-arkusza.xlsx
@@ -9659,7 +9659,11 @@
           <t>p43, p30, p49</t>
         </is>
       </c>
-      <c r="U84" t="inlineStr"/>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>/img/produkty/p83-800.webp</t>
+        </is>
+      </c>
       <c r="V84" t="n">
         <v>83</v>
       </c>
@@ -11307,7 +11311,11 @@
           <t>p34, p27</t>
         </is>
       </c>
-      <c r="U99" t="inlineStr"/>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>/img/produkty/p98-800.webp</t>
+        </is>
+      </c>
       <c r="V99" t="n">
         <v>98</v>
       </c>
@@ -11807,7 +11815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F151"/>
+  <dimension ref="A1:F149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15089,24 +15097,32 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>p83</t>
+          <t>p84</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Maison Francis Kurkdjian Oud Satin Mood</t>
+          <t>Nishane Wūlóng Chá</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr"/>
-      <c r="E107" t="inlineStr"/>
+          <t>opis</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>cikawy niuans</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>ciekawy niuans</t>
+        </is>
+      </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>poprawiona literówka albo myślnik (zasady tekstów marki)</t>
         </is>
       </c>
     </row>
@@ -15123,50 +15139,50 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>opis</t>
+          <t>podobne</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>cikawy niuans</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>ciekawy niuans</t>
-        </is>
-      </c>
+          <t>Xerjoff Renaissance -&gt; renaissance</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
-          <t>poprawiona literówka albo myślnik (zasady tekstów marki)</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>p84</t>
+          <t>p85</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Nishane Wūlóng Chá</t>
+          <t>Sospiro Basso</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>podobne</t>
+          <t>sezon</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Xerjoff Renaissance -&gt; renaissance</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr"/>
+          <t>Wiosna, lato, wczesna jesień</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>wiosna, lato, jesień</t>
+        </is>
+      </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>uproszczono do listy pór roku</t>
         </is>
       </c>
     </row>
@@ -15183,50 +15199,50 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>sezon</t>
+          <t>podobne</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Wiosna, lato, wczesna jesień</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>wiosna, lato, jesień</t>
-        </is>
-      </c>
+          <t>Terre d'Hermes -&gt; terre d'hermes</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
-          <t>uproszczono do listy pór roku</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>p85</t>
+          <t>p88</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Sospiro Basso</t>
+          <t>Tom Ford Oud Voyager</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>podobne</t>
+          <t>opis</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Terre d'Hermes -&gt; terre d'hermes</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr"/>
+          <t>Premiera jest z tego roku</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Premiera była we wrześniu 2025 roku</t>
+        </is>
+      </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>nieaktualna informacja: Oud Voyager jest w sklepach od września 2025, nie z 2026</t>
         </is>
       </c>
     </row>
@@ -15243,22 +15259,22 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>opis</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Premiera jest z tego roku</t>
+          <t>pewność danych: średnia</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Premiera była we wrześniu 2025 roku</t>
+          <t>bez zmian</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>nieaktualna informacja: Oud Voyager jest w sklepach od września 2025, nie z 2026</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
@@ -15275,66 +15291,66 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>pora</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
+          <t>Wieczór (w dzień przy lekkiej aplikacji)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>bez zmian</t>
+          <t>uniwersalna</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>uproszczono do: dzień, wieczór, uniwersalna</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>p88</t>
+          <t>p90</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Tom Ford Oud Voyager</t>
+          <t>Kilian Angels' Share On The Rocks</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>pora</t>
+          <t>opis</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Wieczór (w dzień przy lekkiej aplikacji)</t>
+          <t>gdyznasz</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>uniwersalna</t>
+          <t>gdy znasz</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>uproszczono do: dzień, wieczór, uniwersalna</t>
+          <t>poprawiona literówka albo myślnik (zasady tekstów marki)</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>p90</t>
+          <t>p91</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Kilian Angels' Share On The Rocks</t>
+          <t>Kilian Roses On Ice</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -15344,12 +15360,12 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>gdyznasz</t>
+          <t>wieczorem zaś - piękny alkoholowy akcent</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>gdy znasz</t>
+          <t>wieczorem zaś piękny, alkoholowy akcent</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -15361,12 +15377,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>p91</t>
+          <t>p93</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Kilian Roses On Ice</t>
+          <t>Kilian Good girl gone Bad</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -15376,12 +15392,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>wieczorem zaś - piękny alkoholowy akcent</t>
+          <t>Zpach uniwersalny lecz</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>wieczorem zaś piękny, alkoholowy akcent</t>
+          <t>Zapach uniwersalny, lecz</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -15393,12 +15409,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>p93</t>
+          <t>p94</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Kilian Good girl gone Bad</t>
+          <t>Kilian Sparkling Royal</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -15408,12 +15424,12 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Zpach uniwersalny lecz</t>
+          <t>zyskuje.Zapach</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Zapach uniwersalny, lecz</t>
+          <t>zyskuje. Zapach</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -15435,22 +15451,22 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>opis</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>zyskuje.Zapach</t>
+          <t>pewność danych: średnia</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>zyskuje. Zapach</t>
+          <t>bez zmian</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>poprawiona literówka albo myślnik (zasady tekstów marki)</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
@@ -15467,62 +15483,62 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>podobne</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>bez zmian</t>
-        </is>
-      </c>
+          <t>Xerjoff Renaissance -&gt; renaissance</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>p94</t>
+          <t>p95</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Kilian Sparkling Royal</t>
+          <t>Atkinsons Shine Despite Everything</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>podobne</t>
+          <t>opis</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Xerjoff Renaissance -&gt; renaissance</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr"/>
+          <t>akcentami  kremowości</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>akcentami kremowości</t>
+        </is>
+      </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>poprawiona literówka albo myślnik (zasady tekstów marki)</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>p96</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Atkinsons Shine Despite Everything</t>
+          <t>Atkinsons Oud Save the King</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -15532,12 +15548,12 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>akcentami  kremowości</t>
+          <t>Earl Greyspotyka</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>akcentami kremowości</t>
+          <t>Earl Grey spotyka</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -15549,44 +15565,44 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>p96</t>
+          <t>p97</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Atkinsons Oud Save the King</t>
+          <t>Atkinsons Mint &amp; Tonic</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>opis</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Earl Greyspotyka</t>
+          <t>pewność danych: średnia</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Earl Grey spotyka</t>
+          <t>bez zmian</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>poprawiona literówka albo myślnik (zasady tekstów marki)</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>p97</t>
+          <t>p98</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Atkinsons Mint &amp; Tonic</t>
+          <t>Bohoboco Wet Cherry Liquor</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -15623,122 +15639,130 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>pewność danych: średnia</t>
+          <t>Owocowo-gourmand, w bazie drzewno-waniliowa</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>bez zmian</t>
+          <t>gourmand</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>p98</t>
+          <t>p99</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Bohoboco Wet Cherry Liquor</t>
+          <t>Sisley Soir d'Orient</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>rodzina</t>
+          <t>opis</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Owocowo-gourmand, w bazie drzewno-waniliowa</t>
+          <t>elegankiej</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>gourmand</t>
+          <t>eleganckiej</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>poprawiona literówka albo myślnik (zasady tekstów marki)</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>p98</t>
+          <t>p99</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Bohoboco Wet Cherry Liquor</t>
+          <t>Sisley Soir d'Orient</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>zdjecie_url</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr"/>
-      <c r="E126" t="inlineStr"/>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Przyprawowo-drzewna</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>drzewna</t>
+        </is>
+      </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>brak zdjęcia: strona producenta blokuje pobieranie, potrzebne własne albo prasowe</t>
+          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>p99</t>
+          <t>p100</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Sisley Soir d'Orient</t>
+          <t>Bohoboco Vanilla Black Pepper</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>opis</t>
+          <t>nuty / osiągi</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>elegankiej</t>
+          <t>pewność danych: średnia</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>eleganckiej</t>
+          <t>bez zmian</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>poprawiona literówka albo myślnik (zasady tekstów marki)</t>
+          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>p99</t>
+          <t>p100</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Sisley Soir d'Orient</t>
+          <t>Bohoboco Vanilla Black Pepper</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -15748,12 +15772,12 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Przyprawowo-drzewna</t>
+          <t>Korzenno-waniliowa, ambrowa</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>drzewna</t>
+          <t>ambrowa</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -15765,112 +15789,108 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>p100</t>
+          <t>z01</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Bohoboco Vanilla Black Pepper</t>
+          <t>LV DISCOVERY SET</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>nuty / osiągi</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>pewność danych: średnia</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>bez zmian</t>
-        </is>
-      </c>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr"/>
+      <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
-          <t>instrukcja arkusza: zweryfikować przed publikacją</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>p100</t>
+          <t>z01</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Bohoboco Vanilla Black Pepper</t>
+          <t>LV DISCOVERY SET</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>Korzenno-waniliowa, ambrowa</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>ambrowa</t>
-        </is>
-      </c>
+          <t>opis</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr"/>
+      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
-          <t>pierwszy człon spoza 12 rodzin kanonicznych, propozycja</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>z01</t>
+          <t>z02</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>LV DISCOVERY SET</t>
+          <t>XERJOFF DISCOVERY SET</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr"/>
-      <c r="E131" t="inlineStr"/>
+          <t>sklad</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>5 × 5 ml (do ustalenia skład, sugerowane: Torino21, Renaissance, Erba Pura, Uden, Naxos)</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>p06:5, p07:5, p08:5, p09:5, p10:5</t>
+        </is>
+      </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
+          <t>skład „do ustalenia”; wpisano propozycję ze źródła, zestaw wyłączony</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>z01</t>
+          <t>z02</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>LV DISCOVERY SET</t>
+          <t>XERJOFF DISCOVERY SET</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>opis</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr"/>
+          <t>sklad</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Renaissance -&gt; renaissance</t>
+        </is>
+      </c>
       <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
@@ -15887,22 +15907,14 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>sklad</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>5 × 5 ml (do ustalenia skład, sugerowane: Torino21, Renaissance, Erba Pura, Uden, Naxos)</t>
-        </is>
-      </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>p06:5, p07:5, p08:5, p09:5, p10:5</t>
-        </is>
-      </c>
+          <t>rodzina</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr"/>
+      <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr">
         <is>
-          <t>skład „do ustalenia”; wpisano propozycję ze źródła, zestaw wyłączony</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
@@ -15919,66 +15931,70 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>sklad</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr">
-        <is>
-          <t>Renaissance -&gt; renaissance</t>
-        </is>
-      </c>
+          <t>opis</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr"/>
       <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>z02</t>
+          <t>z03</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>XERJOFF DISCOVERY SET</t>
+          <t>NOUS TOUS DISCOVERY SET</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr"/>
-      <c r="E135" t="inlineStr"/>
+          <t>cena</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>350 zł</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
+          <t>cena zapisana jako tekst</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>z02</t>
+          <t>z03</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>XERJOFF DISCOVERY SET</t>
+          <t>NOUS TOUS DISCOVERY SET</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>opis</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D136" t="inlineStr"/>
       <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
@@ -15995,70 +16011,74 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>cena</t>
-        </is>
-      </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>350 zł</t>
-        </is>
-      </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
+          <t>opis</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr">
         <is>
-          <t>cena zapisana jako tekst</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>z03</t>
+          <t>z04</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>NOUS TOUS DISCOVERY SET</t>
+          <t>SWEET &amp; SPICY SET</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr"/>
-      <c r="E138" t="inlineStr"/>
+          <t>sklad</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>p34</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>p98</t>
+        </is>
+      </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
+          <t>zamiana na prośbę właściciela: zestaw ma być dostępny, a składnik ze źródła jest niedostępny</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>z03</t>
+          <t>z04</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>NOUS TOUS DISCOVERY SET</t>
+          <t>SWEET &amp; SPICY SET</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>opis</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D139" t="inlineStr"/>
-      <c r="E139" t="inlineStr"/>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>gourmand</t>
+        </is>
+      </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
+          <t>propozycja z opisu zestawu w źródle (gourmand wprost w treści)</t>
         </is>
       </c>
     </row>
@@ -16075,74 +16095,66 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>sklad</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>p34</t>
-        </is>
-      </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>p98</t>
-        </is>
-      </c>
+          <t>opis</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
-          <t>zamiana na prośbę właściciela: zestaw ma być dostępny, a składnik ze źródła jest niedostępny</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>z04</t>
+          <t>z05</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>SWEET &amp; SPICY SET</t>
+          <t>ENTRY SET</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr"/>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>gourmand</t>
-        </is>
-      </c>
+          <t>sklad</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Amouage Reflection -&gt; reflection</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr">
         <is>
-          <t>propozycja z opisu zestawu w źródle (gourmand wprost w treści)</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>z04</t>
+          <t>z05</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>SWEET &amp; SPICY SET</t>
+          <t>ENTRY SET</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>opis</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D142" t="inlineStr"/>
       <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
@@ -16159,66 +16171,66 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>sklad</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>Amouage Reflection -&gt; reflection</t>
-        </is>
-      </c>
+          <t>opis</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr"/>
       <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>z05</t>
+          <t>z06</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>ENTRY SET</t>
+          <t>AUTUMN DISCOVERY SET</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr"/>
+          <t>sklad</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>YSL Y le Parfum -&gt; y le parfum</t>
+        </is>
+      </c>
       <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr">
         <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
+          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>z05</t>
+          <t>z06</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>ENTRY SET</t>
+          <t>AUTUMN DISCOVERY SET</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>opis</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D145" t="inlineStr"/>
       <c r="E145" t="inlineStr"/>
       <c r="F145" t="inlineStr">
         <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
@@ -16235,66 +16247,70 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>sklad</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>YSL Y le Parfum -&gt; y le parfum</t>
-        </is>
-      </c>
+          <t>opis</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr"/>
       <c r="E146" t="inlineStr"/>
       <c r="F146" t="inlineStr">
         <is>
-          <t>dopasowano po poprawce literówki albo skrótu nazwy</t>
+          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>z06</t>
+          <t>z07</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>AUTUMN DISCOVERY SET</t>
+          <t>WINTER DISCOVERY SET</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr"/>
-      <c r="E147" t="inlineStr"/>
+          <t>sklad</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>5x ml (BOSS Bottled Absolu, MFK Grand Soir, Maison Crivelli Oud Maracuja, Tom Ford Tobacco Vanille, Montale Arabians Tonka)</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>p60:5, p42:5, p41:5, p35:5, p28:5</t>
+        </is>
+      </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
+          <t>w źródle „5x ml” bez pojemności; przyjęto 5 ml</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>z06</t>
+          <t>z07</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>AUTUMN DISCOVERY SET</t>
+          <t>WINTER DISCOVERY SET</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>opis</t>
+          <t>rodzina</t>
         </is>
       </c>
       <c r="D148" t="inlineStr"/>
       <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr">
         <is>
-          <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
+          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
         </is>
       </c>
     </row>
@@ -16311,68 +16327,12 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>sklad</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>5x ml (BOSS Bottled Absolu, MFK Grand Soir, Maison Crivelli Oud Maracuja, Tom Ford Tobacco Vanille, Montale Arabians Tonka)</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>p60:5, p42:5, p41:5, p35:5, p28:5</t>
-        </is>
-      </c>
+          <t>opis</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr">
-        <is>
-          <t>w źródle „5x ml” bez pojemności; przyjęto 5 ml</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>z07</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>WINTER DISCOVERY SET</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>rodzina</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr"/>
-      <c r="E150" t="inlineStr"/>
-      <c r="F150" t="inlineStr">
-        <is>
-          <t>brak rodziny: quiz nie zaproponuje tego zestawu</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>z07</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>WINTER DISCOVERY SET</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>opis</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr"/>
-      <c r="E151" t="inlineStr"/>
-      <c r="F151" t="inlineStr">
         <is>
           <t>źródło ma tylko opis pozycjonowania dla doradcy; opis dla klienta do napisania</t>
         </is>

</xml_diff>